<commit_message>
Sostituisce Pi Zero 2 W con Pi 4 e doppio buck dedicato (Pi/rele)
Il Pi Zero 2 W si e danneggiato al primo tentativo di accensione della
revisione a rele, probabilmente per una sovratensione sul buck condiviso
tra Pi e bobine del rele. Fix: Raspberry Pi 4 (stesso GPIO a 40 pin,
nessuna modifica al software) e due buck 12V->5V distinti, uno dedicato
al Pi e uno solo per JD-VCC del modulo rele. Aggiornati schemi, lista
spesa e README con checklist di accensione obbligatoria.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/balcony-irrigation-shopping-list/lista_spesa_irrigazione_balcone.xlsx
+++ b/outputs/balcony-irrigation-shopping-list/lista_spesa_irrigazione_balcone.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lista spesa" sheetId="1" r:id="Re0ab505d015b4a3b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Riepilogo" sheetId="2" r:id="Ra10c9d603de34cca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Schema tecnico" sheetId="3" r:id="R5b8e85482cc8495b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lista spesa" sheetId="1" r:id="R662798fdb8e74fba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Riepilogo" sheetId="2" r:id="R1b246cacf47f420e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Schema tecnico" sheetId="3" r:id="R6892b754877241b5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -203,7 +203,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ShoppingList" displayName="ShoppingList" ref="A4:K31" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ShoppingList" displayName="ShoppingList" ref="A4:K32" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Categoria"/>
     <x:tableColumn id="2" name="Priorita"/>
@@ -518,24 +518,24 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D5" s="12" t="str">
-        <x:v>Raspberry Pi Zero 2 WH</x:v>
+        <x:v>Raspberry Pi 4 Model B</x:v>
       </x:c>
       <x:c r="E5" s="12" t="str">
-        <x:v>Zero 2 W with headers / WH, Wi-Fi integrato</x:v>
+        <x:v>4GB o 8GB RAM, Wi-Fi integrato</x:v>
       </x:c>
       <x:c r="F5" s="12" t="str">
-        <x:v>Melopero, The Pi Hut, Welectron</x:v>
+        <x:v>Amazon, Melopero, The Pi Hut</x:v>
       </x:c>
       <x:c r="G5" s="12" t="str">
         <x:v>Da acquistare</x:v>
       </x:c>
       <x:c r="H5" s="15" t="str"/>
       <x:c r="I5" s="14" t="n">
-        <x:v>25</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="J5" s="14" t="str"/>
       <x:c r="K5" s="12" t="str">
-        <x:v>Versione con header gia saldati: niente saldature</x:v>
+        <x:v>Sostituisce il Pi Zero 2 W (guasto): stesso GPIO a 40 pin, nessuna modifica al software</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -580,153 +580,153 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D7" s="12" t="str">
-        <x:v>Convertitore 12V -&gt; 5V</x:v>
+        <x:v>Buck 1: convertitore 12V -&gt; 5V per Pi</x:v>
       </x:c>
       <x:c r="E7" s="12" t="str">
-        <x:v>Buck converter 12V a 5V USB, almeno 3A</x:v>
+        <x:v>XWST o simile, 12V/24V a 5V 5A, protezione sovratensione/cortocircuito/termica</x:v>
       </x:c>
       <x:c r="F7" s="12" t="str">
-        <x:v>Amazon, negozi elettronica</x:v>
+        <x:v>Amazon</x:v>
       </x:c>
       <x:c r="G7" s="12" t="str">
         <x:v>Da acquistare</x:v>
       </x:c>
       <x:c r="H7" s="15" t="str"/>
       <x:c r="I7" s="14" t="n">
-        <x:v>10</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="J7" s="14" t="str"/>
       <x:c r="K7" s="12" t="str">
-        <x:v>Alimenta il Raspberry dalla batteria 12V</x:v>
+        <x:v>Dedicato al Raspberry Pi 4 (richiede 5V/3A): margine sopra il minimo, non condiviso col rele</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="12" t="str">
-        <x:v>Pompe</x:v>
+        <x:v>Alimentazione</x:v>
       </x:c>
       <x:c r="B8" s="12" t="str">
         <x:v>Alta</x:v>
       </x:c>
       <x:c r="C8" s="13" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D8" s="12" t="str">
-        <x:v>Pompa sommersa 12V</x:v>
+        <x:v>Buck 2: convertitore 12V -&gt; 5V per rele</x:v>
       </x:c>
       <x:c r="E8" s="12" t="str">
-        <x:v>Pompa 12V DC circa 600 L/h, prevalenza circa 5 m</x:v>
+        <x:v>12V a 5V 3A fisso, protezione cortocircuito</x:v>
       </x:c>
       <x:c r="F8" s="12" t="str">
-        <x:v>Leroy Merlin, ManoMano, Amazon</x:v>
+        <x:v>Amazon</x:v>
       </x:c>
       <x:c r="G8" s="12" t="str">
         <x:v>Da acquistare</x:v>
       </x:c>
       <x:c r="H8" s="15" t="str"/>
       <x:c r="I8" s="14" t="n">
-        <x:v>12</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="J8" s="14" t="str"/>
       <x:c r="K8" s="12" t="str">
-        <x:v>Una per zona; verificare corrente assorbita</x:v>
+        <x:v>Alimenta solo JD-VCC (bobine rele, circa 210 mA): dedicato, non condiviso col Pi. VCC resta dal 3.3V del Pi</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="12" t="str">
-        <x:v>Elettronica</x:v>
+        <x:v>Pompe</x:v>
       </x:c>
       <x:c r="B9" s="12" t="str">
         <x:v>Alta</x:v>
       </x:c>
       <x:c r="C9" s="13" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D9" s="12" t="str">
-        <x:v>Modulo rele 8 canali 5V optoisolato</x:v>
+        <x:v>Pompa sommersa 12V</x:v>
       </x:c>
       <x:c r="E9" s="12" t="str">
-        <x:v>Elegoo 8-Channel, optoisolato, 10A 250VAC/30VDC, jumper VCC/JD-VCC removibile</x:v>
+        <x:v>Pompa 12V DC circa 600 L/h, prevalenza circa 5 m</x:v>
       </x:c>
       <x:c r="F9" s="12" t="str">
-        <x:v>Amazon (Elegoo)</x:v>
+        <x:v>Leroy Merlin, ManoMano, Amazon</x:v>
       </x:c>
       <x:c r="G9" s="12" t="str">
         <x:v>Da acquistare</x:v>
       </x:c>
       <x:c r="H9" s="15" t="str"/>
       <x:c r="I9" s="14" t="n">
-        <x:v>10</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="J9" s="14" t="str"/>
       <x:c r="K9" s="12" t="str">
-        <x:v>Sostituisce i driver MOSFET (calo di tensione sui cavetti JST sotto carico): usa 3 canali su 8, margine per espansioni</x:v>
+        <x:v>Una per zona; verificare corrente assorbita</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="12" t="str">
-        <x:v>Protezione</x:v>
+        <x:v>Elettronica</x:v>
       </x:c>
       <x:c r="B10" s="12" t="str">
         <x:v>Alta</x:v>
       </x:c>
       <x:c r="C10" s="13" t="n">
-        <x:v>5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D10" s="12" t="str">
-        <x:v>Diodo di ricircolo</x:v>
+        <x:v>Modulo rele 8 canali 5V optoisolato</x:v>
       </x:c>
       <x:c r="E10" s="12" t="str">
-        <x:v>1N5819 Schottky (o 1N4007)</x:v>
+        <x:v>Elegoo 8-Channel, optoisolato, 10A 250VAC/30VDC, jumper VCC/JD-VCC removibile</x:v>
       </x:c>
       <x:c r="F10" s="12" t="str">
-        <x:v>Amazon, negozi elettronica</x:v>
+        <x:v>Amazon (Elegoo)</x:v>
       </x:c>
       <x:c r="G10" s="12" t="str">
         <x:v>Da acquistare</x:v>
       </x:c>
       <x:c r="H10" s="15" t="str"/>
       <x:c r="I10" s="14" t="n">
-        <x:v>1</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="J10" s="14" t="str"/>
       <x:c r="K10" s="12" t="str">
-        <x:v>Uno in antiparallelo su ogni pompa, catodo al +: assorbe lo spike induttivo quando il rele apre</x:v>
+        <x:v>Sostituisce i driver MOSFET (calo di tensione sui cavetti JST sotto carico): usa 3 canali su 8, margine per espansioni</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="12" t="str">
-        <x:v>Cablaggio</x:v>
+        <x:v>Protezione</x:v>
       </x:c>
       <x:c r="B11" s="12" t="str">
         <x:v>Alta</x:v>
       </x:c>
       <x:c r="C11" s="13" t="n">
-        <x:v>1</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D11" s="12" t="str">
-        <x:v>Jumper Dupont femmina-femmina</x:v>
+        <x:v>Diodo di ricircolo</x:v>
       </x:c>
       <x:c r="E11" s="12" t="str">
-        <x:v>Kit 40 pin F-F, 10-20 cm</x:v>
+        <x:v>1N5819 Schottky (o 1N4007)</x:v>
       </x:c>
       <x:c r="F11" s="12" t="str">
-        <x:v>Amazon</x:v>
+        <x:v>Amazon, negozi elettronica</x:v>
       </x:c>
       <x:c r="G11" s="12" t="str">
         <x:v>Da acquistare</x:v>
       </x:c>
       <x:c r="H11" s="15" t="str"/>
       <x:c r="I11" s="14" t="n">
-        <x:v>5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J11" s="14" t="str"/>
       <x:c r="K11" s="12" t="str">
-        <x:v>IN1/IN2/IN3, VCC, JD-VCC, GND della scheda rele verso i pin header del Raspberry</x:v>
+        <x:v>Uno in antiparallelo su ogni pompa, catodo al +: assorbe lo spike induttivo quando il rele apre</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="12" t="str">
-        <x:v>Alimentazione</x:v>
+        <x:v>Cablaggio</x:v>
       </x:c>
       <x:c r="B12" s="12" t="str">
         <x:v>Alta</x:v>
@@ -735,29 +735,29 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D12" s="12" t="str">
-        <x:v>Batteria LiFePO4 12V</x:v>
+        <x:v>Jumper Dupont femmina-femmina</x:v>
       </x:c>
       <x:c r="E12" s="12" t="str">
-        <x:v>12.8V 20Ah con BMS integrato</x:v>
+        <x:v>Kit 40 pin F-F, 10-20 cm</x:v>
       </x:c>
       <x:c r="F12" s="12" t="str">
-        <x:v>Amazon: ECO-WORTHY, Renogy, Redodo, Kepworth</x:v>
+        <x:v>Amazon</x:v>
       </x:c>
       <x:c r="G12" s="12" t="str">
         <x:v>Da acquistare</x:v>
       </x:c>
       <x:c r="H12" s="15" t="str"/>
       <x:c r="I12" s="14" t="n">
-        <x:v>75</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="J12" s="14" t="str"/>
       <x:c r="K12" s="12" t="str">
-        <x:v>20Ah consigliati per margine</x:v>
+        <x:v>IN1/IN2/IN3, VCC, JD-VCC, GND della scheda rele verso i pin header del Raspberry</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="12" t="str">
-        <x:v>Solare</x:v>
+        <x:v>Alimentazione</x:v>
       </x:c>
       <x:c r="B13" s="12" t="str">
         <x:v>Alta</x:v>
@@ -766,24 +766,24 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D13" s="12" t="str">
-        <x:v>Regolatore solare MPPT</x:v>
+        <x:v>Batteria LiFePO4 12V</x:v>
       </x:c>
       <x:c r="E13" s="12" t="str">
-        <x:v>Victron SmartSolar MPPT 75/10 compatibile LiFePO4</x:v>
+        <x:v>12.8V 20Ah con BMS integrato</x:v>
       </x:c>
       <x:c r="F13" s="12" t="str">
-        <x:v>Moory, Toosolar, Amazon</x:v>
+        <x:v>Amazon: ECO-WORTHY, Renogy, Redodo, Kepworth</x:v>
       </x:c>
       <x:c r="G13" s="12" t="str">
         <x:v>Da acquistare</x:v>
       </x:c>
       <x:c r="H13" s="15" t="str"/>
       <x:c r="I13" s="14" t="n">
-        <x:v>70</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="J13" s="14" t="str"/>
       <x:c r="K13" s="12" t="str">
-        <x:v>Piu affidabile dei PWM economici</x:v>
+        <x:v>20Ah consigliati per margine</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -797,29 +797,29 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D14" s="12" t="str">
-        <x:v>Pannello solare</x:v>
+        <x:v>Regolatore solare MPPT</x:v>
       </x:c>
       <x:c r="E14" s="12" t="str">
-        <x:v>Pannello 12V 50W minimo, 100W consigliato</x:v>
+        <x:v>Victron SmartSolar MPPT 75/10 compatibile LiFePO4</x:v>
       </x:c>
       <x:c r="F14" s="12" t="str">
-        <x:v>FuturaNet, Amazon, Leroy Merlin</x:v>
+        <x:v>Moory, Toosolar, Amazon</x:v>
       </x:c>
       <x:c r="G14" s="12" t="str">
         <x:v>Da acquistare</x:v>
       </x:c>
       <x:c r="H14" s="15" t="str"/>
       <x:c r="I14" s="14" t="n">
-        <x:v>65</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="J14" s="14" t="str"/>
       <x:c r="K14" s="12" t="str">
-        <x:v>100W se vuoi piu autonomia in giorni nuvolosi</x:v>
+        <x:v>Piu affidabile dei PWM economici</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="12" t="str">
-        <x:v>Idraulica</x:v>
+        <x:v>Solare</x:v>
       </x:c>
       <x:c r="B15" s="12" t="str">
         <x:v>Alta</x:v>
@@ -828,24 +828,24 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D15" s="12" t="str">
-        <x:v>Kit irrigazione balcone</x:v>
+        <x:v>Pannello solare</x:v>
       </x:c>
       <x:c r="E15" s="12" t="str">
-        <x:v>Claber Kit Terrazzo 90772 o Kit Drip 20 vasi 90764</x:v>
+        <x:v>Pannello 12V 50W minimo, 100W consigliato</x:v>
       </x:c>
       <x:c r="F15" s="12" t="str">
-        <x:v>Claber, Leroy Merlin, Brico, ManoMano</x:v>
+        <x:v>FuturaNet, Amazon, Leroy Merlin</x:v>
       </x:c>
       <x:c r="G15" s="12" t="str">
         <x:v>Da acquistare</x:v>
       </x:c>
       <x:c r="H15" s="15" t="str"/>
       <x:c r="I15" s="14" t="n">
-        <x:v>55</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="J15" s="14" t="str"/>
       <x:c r="K15" s="12" t="str">
-        <x:v>Da dividere in tre zone separate</x:v>
+        <x:v>100W se vuoi piu autonomia in giorni nuvolosi</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -856,27 +856,27 @@
         <x:v>Alta</x:v>
       </x:c>
       <x:c r="C16" s="13" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D16" s="12" t="str">
-        <x:v>Valvola di non ritorno</x:v>
+        <x:v>Kit irrigazione balcone</x:v>
       </x:c>
       <x:c r="E16" s="12" t="str">
-        <x:v>Valvola per tubo 6/8/10 mm secondo diametro pompa</x:v>
+        <x:v>Claber Kit Terrazzo 90772 o Kit Drip 20 vasi 90764</x:v>
       </x:c>
       <x:c r="F16" s="12" t="str">
-        <x:v>Amazon, negozi acquari, Leroy Merlin</x:v>
+        <x:v>Claber, Leroy Merlin, Brico, ManoMano</x:v>
       </x:c>
       <x:c r="G16" s="12" t="str">
         <x:v>Da acquistare</x:v>
       </x:c>
       <x:c r="H16" s="15" t="str"/>
       <x:c r="I16" s="14" t="n">
-        <x:v>3</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="J16" s="14" t="str"/>
       <x:c r="K16" s="12" t="str">
-        <x:v>Una dopo ogni pompa</x:v>
+        <x:v>Da dividere in tre zone separate</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -890,24 +890,24 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="D17" s="12" t="str">
-        <x:v>Filtro in linea</x:v>
+        <x:v>Valvola di non ritorno</x:v>
       </x:c>
       <x:c r="E17" s="12" t="str">
-        <x:v>Filtro microirrigazione 120/150 mesh</x:v>
+        <x:v>Valvola per tubo 6/8/10 mm secondo diametro pompa</x:v>
       </x:c>
       <x:c r="F17" s="12" t="str">
-        <x:v>Amazon, agrarie, Leroy Merlin</x:v>
+        <x:v>Amazon, negozi acquari, Leroy Merlin</x:v>
       </x:c>
       <x:c r="G17" s="12" t="str">
         <x:v>Da acquistare</x:v>
       </x:c>
       <x:c r="H17" s="15" t="str"/>
       <x:c r="I17" s="14" t="n">
-        <x:v>5</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="J17" s="14" t="str"/>
       <x:c r="K17" s="12" t="str">
-        <x:v>Riduce intasamento gocciolatori</x:v>
+        <x:v>Una dopo ogni pompa</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -918,32 +918,32 @@
         <x:v>Alta</x:v>
       </x:c>
       <x:c r="C18" s="13" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D18" s="12" t="str">
-        <x:v>Serbatoio acqua</x:v>
+        <x:v>Filtro in linea</x:v>
       </x:c>
       <x:c r="E18" s="12" t="str">
-        <x:v>60-100 L, opaco, con coperchio</x:v>
+        <x:v>Filtro microirrigazione 120/150 mesh</x:v>
       </x:c>
       <x:c r="F18" s="12" t="str">
-        <x:v>Leroy Merlin, Brico, agrarie</x:v>
+        <x:v>Amazon, agrarie, Leroy Merlin</x:v>
       </x:c>
       <x:c r="G18" s="12" t="str">
         <x:v>Da acquistare</x:v>
       </x:c>
       <x:c r="H18" s="15" t="str"/>
       <x:c r="I18" s="14" t="n">
-        <x:v>35</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="J18" s="14" t="str"/>
       <x:c r="K18" s="12" t="str">
-        <x:v>Meglio in ombra e chiuso</x:v>
+        <x:v>Riduce intasamento gocciolatori</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="12" t="str">
-        <x:v>Protezione</x:v>
+        <x:v>Idraulica</x:v>
       </x:c>
       <x:c r="B19" s="12" t="str">
         <x:v>Alta</x:v>
@@ -952,24 +952,24 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D19" s="12" t="str">
-        <x:v>Scatola elettrica stagna</x:v>
+        <x:v>Serbatoio acqua</x:v>
       </x:c>
       <x:c r="E19" s="12" t="str">
-        <x:v>Box IP65/IP66 circa 190x140x70 mm o piu grande</x:v>
+        <x:v>60-100 L, opaco, con coperchio</x:v>
       </x:c>
       <x:c r="F19" s="12" t="str">
-        <x:v>Leroy Merlin, Amazon, elettricista</x:v>
+        <x:v>Leroy Merlin, Brico, agrarie</x:v>
       </x:c>
       <x:c r="G19" s="12" t="str">
         <x:v>Da acquistare</x:v>
       </x:c>
       <x:c r="H19" s="15" t="str"/>
       <x:c r="I19" s="14" t="n">
-        <x:v>15</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="J19" s="14" t="str"/>
       <x:c r="K19" s="12" t="str">
-        <x:v>Tenere in ombra o schermata dal sole diretto</x:v>
+        <x:v>Meglio in ombra e chiuso</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -983,29 +983,29 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D20" s="12" t="str">
-        <x:v>Set pressacavi</x:v>
+        <x:v>Scatola elettrica stagna</x:v>
       </x:c>
       <x:c r="E20" s="12" t="str">
-        <x:v>Pressacavi IP68 M12/M16 assortiti</x:v>
+        <x:v>Box IP65/IP66 almeno 220x170x90 mm (Pi 4 piu ingombrante dello Zero)</x:v>
       </x:c>
       <x:c r="F20" s="12" t="str">
-        <x:v>Amazon, Leroy Merlin</x:v>
+        <x:v>Leroy Merlin, Amazon, elettricista</x:v>
       </x:c>
       <x:c r="G20" s="12" t="str">
         <x:v>Da acquistare</x:v>
       </x:c>
       <x:c r="H20" s="15" t="str"/>
       <x:c r="I20" s="14" t="n">
-        <x:v>10</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="J20" s="14" t="str"/>
       <x:c r="K20" s="12" t="str">
-        <x:v>Per ingressi cavi nel box</x:v>
+        <x:v>Tenere in ombra o schermata dal sole diretto; verifica che ci stiano Pi 4 + due buck + scheda rele</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="12" t="str">
-        <x:v>Cablaggio</x:v>
+        <x:v>Protezione</x:v>
       </x:c>
       <x:c r="B21" s="12" t="str">
         <x:v>Alta</x:v>
@@ -1014,24 +1014,24 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D21" s="12" t="str">
-        <x:v>Morsetti Wago 221</x:v>
+        <x:v>Set pressacavi</x:v>
       </x:c>
       <x:c r="E21" s="12" t="str">
-        <x:v>Set Wago 221 2/3/5 poli</x:v>
+        <x:v>Pressacavi IP68 M12/M16 assortiti</x:v>
       </x:c>
       <x:c r="F21" s="12" t="str">
-        <x:v>Amazon, elettricista</x:v>
+        <x:v>Amazon, Leroy Merlin</x:v>
       </x:c>
       <x:c r="G21" s="12" t="str">
         <x:v>Da acquistare</x:v>
       </x:c>
       <x:c r="H21" s="15" t="str"/>
       <x:c r="I21" s="14" t="n">
-        <x:v>15</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="J21" s="14" t="str"/>
       <x:c r="K21" s="12" t="str">
-        <x:v>Per evitare saldature</x:v>
+        <x:v>Per ingressi cavi nel box</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -1042,27 +1042,27 @@
         <x:v>Alta</x:v>
       </x:c>
       <x:c r="C22" s="13" t="n">
-        <x:v>5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D22" s="12" t="str">
-        <x:v>Portafusibili 12V</x:v>
+        <x:v>Morsetti Wago 221</x:v>
       </x:c>
       <x:c r="E22" s="12" t="str">
-        <x:v>Portafusibili auto ATO/ATC impermeabili</x:v>
+        <x:v>Set Wago 221 2/3/5 poli</x:v>
       </x:c>
       <x:c r="F22" s="12" t="str">
-        <x:v>Amazon, autoricambi</x:v>
+        <x:v>Amazon, elettricista</x:v>
       </x:c>
       <x:c r="G22" s="12" t="str">
         <x:v>Da acquistare</x:v>
       </x:c>
       <x:c r="H22" s="15" t="str"/>
       <x:c r="I22" s="14" t="n">
-        <x:v>2</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="J22" s="14" t="str"/>
       <x:c r="K22" s="12" t="str">
-        <x:v>Generale + uno per ogni pompa + scorta</x:v>
+        <x:v>Per evitare saldature</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -1073,13 +1073,13 @@
         <x:v>Alta</x:v>
       </x:c>
       <x:c r="C23" s="13" t="n">
-        <x:v>1</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D23" s="12" t="str">
-        <x:v>Set fusibili</x:v>
+        <x:v>Portafusibili 12V</x:v>
       </x:c>
       <x:c r="E23" s="12" t="str">
-        <x:v>Fusibili auto 2A/3A/5A/10A assortiti</x:v>
+        <x:v>Portafusibili auto ATO/ATC impermeabili</x:v>
       </x:c>
       <x:c r="F23" s="12" t="str">
         <x:v>Amazon, autoricambi</x:v>
@@ -1089,11 +1089,11 @@
       </x:c>
       <x:c r="H23" s="15" t="str"/>
       <x:c r="I23" s="14" t="n">
-        <x:v>8</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J23" s="14" t="str"/>
       <x:c r="K23" s="12" t="str">
-        <x:v>Dimensionare in base alle pompe reali</x:v>
+        <x:v>Generale + uno per ogni pompa + scorta</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -1101,19 +1101,19 @@
         <x:v>Cablaggio</x:v>
       </x:c>
       <x:c r="B24" s="12" t="str">
-        <x:v>Media</x:v>
+        <x:v>Alta</x:v>
       </x:c>
       <x:c r="C24" s="13" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D24" s="12" t="str">
-        <x:v>Interruttore generale 12V</x:v>
+        <x:v>Set fusibili</x:v>
       </x:c>
       <x:c r="E24" s="12" t="str">
-        <x:v>Interruttore DC da quadro o impermeabile</x:v>
+        <x:v>Fusibili auto 2A/3A/5A/10A assortiti</x:v>
       </x:c>
       <x:c r="F24" s="12" t="str">
-        <x:v>Amazon, elettricista</x:v>
+        <x:v>Amazon, autoricambi</x:v>
       </x:c>
       <x:c r="G24" s="12" t="str">
         <x:v>Da acquistare</x:v>
@@ -1124,38 +1124,38 @@
       </x:c>
       <x:c r="J24" s="14" t="str"/>
       <x:c r="K24" s="12" t="str">
-        <x:v>Per manutenzione rapida</x:v>
+        <x:v>Dimensionare in base alle pompe reali</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="12" t="str">
-        <x:v>Sensori</x:v>
+        <x:v>Cablaggio</x:v>
       </x:c>
       <x:c r="B25" s="12" t="str">
-        <x:v>Alta</x:v>
+        <x:v>Media</x:v>
       </x:c>
       <x:c r="C25" s="13" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D25" s="12" t="str">
-        <x:v>Sensore livello acqua</x:v>
+        <x:v>Interruttore generale 12V</x:v>
       </x:c>
       <x:c r="E25" s="12" t="str">
-        <x:v>Galleggiante serbatoio NO/NC</x:v>
+        <x:v>Interruttore DC da quadro o impermeabile</x:v>
       </x:c>
       <x:c r="F25" s="12" t="str">
-        <x:v>Amazon, negozi elettronica</x:v>
+        <x:v>Amazon, elettricista</x:v>
       </x:c>
       <x:c r="G25" s="12" t="str">
         <x:v>Da acquistare</x:v>
       </x:c>
       <x:c r="H25" s="15" t="str"/>
       <x:c r="I25" s="14" t="n">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="J25" s="14" t="str"/>
       <x:c r="K25" s="12" t="str">
-        <x:v>Blocco anti-marcia a secco</x:v>
+        <x:v>Per manutenzione rapida</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -1163,30 +1163,30 @@
         <x:v>Sensori</x:v>
       </x:c>
       <x:c r="B26" s="12" t="str">
-        <x:v>Media</x:v>
+        <x:v>Alta</x:v>
       </x:c>
       <x:c r="C26" s="13" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D26" s="12" t="str">
-        <x:v>ADC ADS1115</x:v>
+        <x:v>Sensore livello acqua</x:v>
       </x:c>
       <x:c r="E26" s="12" t="str">
-        <x:v>ADS1115 I2C 16 bit pre-soldered / STEMMA QT</x:v>
+        <x:v>Galleggiante serbatoio NO/NC</x:v>
       </x:c>
       <x:c r="F26" s="12" t="str">
-        <x:v>Adafruit, Amazon, Seeed, Robot Italy</x:v>
+        <x:v>Amazon, negozi elettronica</x:v>
       </x:c>
       <x:c r="G26" s="12" t="str">
         <x:v>Da acquistare</x:v>
       </x:c>
       <x:c r="H26" s="15" t="str"/>
       <x:c r="I26" s="14" t="n">
-        <x:v>12</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="J26" s="14" t="str"/>
       <x:c r="K26" s="12" t="str">
-        <x:v>Serve per sensori analogici umidita</x:v>
+        <x:v>Blocco anti-marcia a secco</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -1197,16 +1197,16 @@
         <x:v>Media</x:v>
       </x:c>
       <x:c r="C27" s="13" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D27" s="12" t="str">
-        <x:v>Sensori umidita terreno</x:v>
+        <x:v>ADC ADS1115</x:v>
       </x:c>
       <x:c r="E27" s="12" t="str">
-        <x:v>DFRobot SEN0308 waterproof capacitivo o equivalente</x:v>
+        <x:v>ADS1115 I2C 16 bit pre-soldered / STEMMA QT</x:v>
       </x:c>
       <x:c r="F27" s="12" t="str">
-        <x:v>Farnell, DFRobot, Robot Italy</x:v>
+        <x:v>Adafruit, Amazon, Seeed, Robot Italy</x:v>
       </x:c>
       <x:c r="G27" s="12" t="str">
         <x:v>Da acquistare</x:v>
@@ -1217,7 +1217,7 @@
       </x:c>
       <x:c r="J27" s="14" t="str"/>
       <x:c r="K27" s="12" t="str">
-        <x:v>Uno per zona all'inizio</x:v>
+        <x:v>Serve per sensori analogici umidita</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -1225,66 +1225,66 @@
         <x:v>Sensori</x:v>
       </x:c>
       <x:c r="B28" s="12" t="str">
-        <x:v>Bassa</x:v>
+        <x:v>Media</x:v>
       </x:c>
       <x:c r="C28" s="13" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D28" s="12" t="str">
-        <x:v>Sensore aria</x:v>
+        <x:v>Sensori umidita terreno</x:v>
       </x:c>
       <x:c r="E28" s="12" t="str">
-        <x:v>BME280 o SHT31 temperatura/umidita</x:v>
+        <x:v>DFRobot SEN0308 waterproof capacitivo o equivalente</x:v>
       </x:c>
       <x:c r="F28" s="12" t="str">
-        <x:v>Amazon, Robot Italy, Melopero</x:v>
+        <x:v>Farnell, DFRobot, Robot Italy</x:v>
       </x:c>
       <x:c r="G28" s="12" t="str">
         <x:v>Da acquistare</x:v>
       </x:c>
       <x:c r="H28" s="15" t="str"/>
       <x:c r="I28" s="14" t="n">
-        <x:v>8</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="J28" s="14" t="str"/>
       <x:c r="K28" s="12" t="str">
-        <x:v>Utile per modalita estate/inverno</x:v>
+        <x:v>Uno per zona all'inizio</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="12" t="str">
-        <x:v>Cablaggio</x:v>
+        <x:v>Sensori</x:v>
       </x:c>
       <x:c r="B29" s="12" t="str">
-        <x:v>Media</x:v>
+        <x:v>Bassa</x:v>
       </x:c>
       <x:c r="C29" s="13" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D29" s="12" t="str">
-        <x:v>Cavo elettrico pompe</x:v>
+        <x:v>Sensore aria</x:v>
       </x:c>
       <x:c r="E29" s="12" t="str">
-        <x:v>2x0.75 mm2 o 2x1 mm2</x:v>
+        <x:v>BME280 o SHT31 temperatura/umidita</x:v>
       </x:c>
       <x:c r="F29" s="12" t="str">
-        <x:v>Leroy Merlin, Brico, elettricista</x:v>
+        <x:v>Amazon, Robot Italy, Melopero</x:v>
       </x:c>
       <x:c r="G29" s="12" t="str">
         <x:v>Da acquistare</x:v>
       </x:c>
       <x:c r="H29" s="15" t="str"/>
       <x:c r="I29" s="14" t="n">
-        <x:v>20</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="J29" s="14" t="str"/>
       <x:c r="K29" s="12" t="str">
-        <x:v>Usare sezioni maggiori per tratte lunghe</x:v>
+        <x:v>Utile per modalita estate/inverno</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="12" t="str">
-        <x:v>Idraulica</x:v>
+        <x:v>Cablaggio</x:v>
       </x:c>
       <x:c r="B30" s="12" t="str">
         <x:v>Media</x:v>
@@ -1293,54 +1293,85 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D30" s="12" t="str">
-        <x:v>Tubi e raccordi extra</x:v>
+        <x:v>Cavo elettrico pompe</x:v>
       </x:c>
       <x:c r="E30" s="12" t="str">
-        <x:v>Microtubo 4/6 mm, tubo 8/10 mm, T, rubinetti, tappi</x:v>
+        <x:v>2x0.75 mm2 o 2x1 mm2</x:v>
       </x:c>
       <x:c r="F30" s="12" t="str">
-        <x:v>Claber, Leroy Merlin, agrarie</x:v>
+        <x:v>Leroy Merlin, Brico, elettricista</x:v>
       </x:c>
       <x:c r="G30" s="12" t="str">
         <x:v>Da acquistare</x:v>
       </x:c>
       <x:c r="H30" s="15" t="str"/>
       <x:c r="I30" s="14" t="n">
-        <x:v>25</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="J30" s="14" t="str"/>
       <x:c r="K30" s="12" t="str">
-        <x:v>Serve sempre piu di quanto sembra</x:v>
+        <x:v>Usare sezioni maggiori per tratte lunghe</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="12" t="str">
-        <x:v>Cablaggio</x:v>
+        <x:v>Idraulica</x:v>
       </x:c>
       <x:c r="B31" s="12" t="str">
         <x:v>Media</x:v>
       </x:c>
       <x:c r="C31" s="13" t="n">
-        <x:v>6</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D31" s="12" t="str">
-        <x:v>Connettori impermeabili 2 pin</x:v>
+        <x:v>Tubi e raccordi extra</x:v>
       </x:c>
       <x:c r="E31" s="12" t="str">
-        <x:v>Connettori IP67/IP68 a vite o pre-cablati</x:v>
+        <x:v>Microtubo 4/6 mm, tubo 8/10 mm, T, rubinetti, tappi</x:v>
       </x:c>
       <x:c r="F31" s="12" t="str">
-        <x:v>Amazon, negozi elettronica</x:v>
+        <x:v>Claber, Leroy Merlin, agrarie</x:v>
       </x:c>
       <x:c r="G31" s="12" t="str">
         <x:v>Da acquistare</x:v>
       </x:c>
       <x:c r="H31" s="15" t="str"/>
       <x:c r="I31" s="14" t="n">
-        <x:v>3</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="J31" s="14" t="str"/>
       <x:c r="K31" s="12" t="str">
+        <x:v>Serve sempre piu di quanto sembra</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="12" t="str">
+        <x:v>Cablaggio</x:v>
+      </x:c>
+      <x:c r="B32" s="12" t="str">
+        <x:v>Media</x:v>
+      </x:c>
+      <x:c r="C32" s="13" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="D32" s="12" t="str">
+        <x:v>Connettori impermeabili 2 pin</x:v>
+      </x:c>
+      <x:c r="E32" s="12" t="str">
+        <x:v>Connettori IP67/IP68 a vite o pre-cablati</x:v>
+      </x:c>
+      <x:c r="F32" s="12" t="str">
+        <x:v>Amazon, negozi elettronica</x:v>
+      </x:c>
+      <x:c r="G32" s="12" t="str">
+        <x:v>Da acquistare</x:v>
+      </x:c>
+      <x:c r="H32" s="15" t="str"/>
+      <x:c r="I32" s="14" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J32" s="14" t="str"/>
+      <x:c r="K32" s="12" t="str">
         <x:v>Per staccare pompe e sensori senza aprire tutto</x:v>
       </x:c>
     </x:row>
@@ -1349,22 +1380,22 @@
     <x:mergeCell ref="A1:K1"/>
     <x:mergeCell ref="A2:K2"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="G5:G31">
+  <x:conditionalFormatting sqref="G5:G32">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Acquistato"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Da acquistare"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Ordinato"/>
   </x:conditionalFormatting>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="G5:G31">
+    <x:dataValidation type="list" sqref="G5:G32">
       <x:formula1>"Da acquistare,Ordinato,Acquistato,Non serve"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="B5:B31">
+    <x:dataValidation type="list" sqref="B5:B32">
       <x:formula1>"Alta,Media,Bassa"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R07fa51bf9172475b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda336532fa3d4e93"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1403,8 +1434,8 @@
         <x:v>Totale righe</x:v>
       </x:c>
       <x:c r="B3" s="12" t="n">
-        <x:f>COUNTA('Lista spesa'!D5:D31)</x:f>
-        <x:v>27</x:v>
+        <x:f>COUNTA('Lista spesa'!D5:D32)</x:f>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="C3" s="24"/>
       <x:c r="D3" s="28" t="str">
@@ -1422,8 +1453,8 @@
         <x:v>Da acquistare</x:v>
       </x:c>
       <x:c r="B4" s="12" t="n">
-        <x:f>COUNTIF('Lista spesa'!G5:G31,"Da acquistare")</x:f>
-        <x:v>27</x:v>
+        <x:f>COUNTIF('Lista spesa'!G5:G32,"Da acquistare")</x:f>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="C4" s="24"/>
       <x:c r="D4" s="12" t="str">
@@ -1441,7 +1472,7 @@
         <x:v>Ordinato</x:v>
       </x:c>
       <x:c r="B5" s="12" t="n">
-        <x:f>COUNTIF('Lista spesa'!G5:G31,"Ordinato")</x:f>
+        <x:f>COUNTIF('Lista spesa'!G5:G32,"Ordinato")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C5" s="24"/>
@@ -1460,7 +1491,7 @@
         <x:v>Acquistato</x:v>
       </x:c>
       <x:c r="B6" s="12" t="n">
-        <x:f>COUNTIF('Lista spesa'!G5:G31,"Acquistato")</x:f>
+        <x:f>COUNTIF('Lista spesa'!G5:G32,"Acquistato")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C6" s="24"/>
@@ -1479,7 +1510,7 @@
         <x:v>Non serve</x:v>
       </x:c>
       <x:c r="B7" s="12" t="n">
-        <x:f>COUNTIF('Lista spesa'!G5:G31,"Non serve")</x:f>
+        <x:f>COUNTIF('Lista spesa'!G5:G32,"Non serve")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C7" s="24"/>
@@ -1498,8 +1529,8 @@
         <x:v>Budget stimato</x:v>
       </x:c>
       <x:c r="B8" s="14" t="n">
-        <x:f>SUMPRODUCT('Lista spesa'!C5:C31,'Lista spesa'!I5:I31)</x:f>
-        <x:v>617</x:v>
+        <x:f>SUMPRODUCT('Lista spesa'!C5:C32,'Lista spesa'!I5:I32)</x:f>
+        <x:v>675</x:v>
       </x:c>
       <x:c r="C8" s="24"/>
       <x:c r="D8" s="12" t="str">
@@ -1686,7 +1717,7 @@
         <x:v>Logica rele</x:v>
       </x:c>
       <x:c r="D8" s="12" t="str">
-        <x:v>Active-low: GPIO basso = rele chiuso = pompa ON. VCC opto da 3.3V Pi, JD-VCC da 5V Pi, jumper rimosso</x:v>
+        <x:v>Active-low: GPIO basso = rele chiuso = pompa ON. Jumper VCC-JD-VCC rimosso</x:v>
       </x:c>
       <x:c r="E8" s="24"/>
       <x:c r="F8" s="12" t="str">
@@ -1698,6 +1729,42 @@
       <x:c r="H8" s="12" t="str">
         <x:v>Poi imposta tempi</x:v>
       </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="12" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B9" s="12" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="C9" s="12" t="str">
+        <x:v>Alimentazione rele</x:v>
+      </x:c>
+      <x:c r="D9" s="12" t="str">
+        <x:v>VCC opto da 3.3V Pi (pin 1); JD-VCC bobine dal Buck 2 dedicato (non dal Pi)</x:v>
+      </x:c>
+      <x:c r="E9" s="24"/>
+      <x:c r="F9" s="24"/>
+      <x:c r="G9" s="24"/>
+      <x:c r="H9" s="24"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="12" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B10" s="12" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="C10" s="12" t="str">
+        <x:v>Alimentazione Pi</x:v>
+      </x:c>
+      <x:c r="D10" s="12" t="str">
+        <x:v>Buck 1 dedicato al Pi 4 (5V/5A): testare sotto carico prima di collegare il Pi</x:v>
+      </x:c>
+      <x:c r="E10" s="24"/>
+      <x:c r="F10" s="24"/>
+      <x:c r="G10" s="24"/>
+      <x:c r="H10" s="24"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>